<commit_message>
ready new paser with guide
</commit_message>
<xml_diff>
--- a/input/timetable/Бизнес-информатика.xlsx
+++ b/input/timetable/Бизнес-информатика.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13890" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13890"/>
   </bookViews>
   <sheets>
     <sheet name="1 курс" sheetId="25" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="121">
   <si>
     <t>пара</t>
   </si>
@@ -70,6 +70,9 @@
     <t>Зав. кафедрой</t>
   </si>
   <si>
+    <t>Преподаватель</t>
+  </si>
+  <si>
     <t>Направление</t>
   </si>
   <si>
@@ -113,6 +116,9 @@
   </si>
   <si>
     <t>ЭУК</t>
+  </si>
+  <si>
+    <t>Попова Е.В.</t>
   </si>
   <si>
     <t>407-31</t>
@@ -122,6 +128,12 @@
 </t>
   </si>
   <si>
+    <t>Лешукова Е.В.</t>
+  </si>
+  <si>
+    <t>Вариясова Е.В.</t>
+  </si>
+  <si>
     <t>407-41</t>
   </si>
   <si>
@@ -137,9 +149,27 @@
     <t>Философия (лек 32 ч)</t>
   </si>
   <si>
+    <t>Бутенко Н.А.</t>
+  </si>
+  <si>
     <t>Работа в команде (лек 32 ч)</t>
   </si>
   <si>
+    <t>Осипова А.В.</t>
+  </si>
+  <si>
+    <t>Курамшина А.В.</t>
+  </si>
+  <si>
+    <t>Заведеев Е.В.</t>
+  </si>
+  <si>
+    <t>Маслов  Н.С.</t>
+  </si>
+  <si>
+    <t>Исаева И.А.</t>
+  </si>
+  <si>
     <t>Начальник УОпоОФО</t>
   </si>
   <si>
@@ -161,15 +191,39 @@
     <t>Экономика предприятий и управление бизнес-процессами                              (ТО: 02.02.2026-06.06.2026)</t>
   </si>
   <si>
+    <t>Ахтемзянова Н.М.</t>
+  </si>
+  <si>
+    <t>Костюнина М.В.; Ситникова А.Ю.</t>
+  </si>
+  <si>
+    <t>Галлямова Л.В.</t>
+  </si>
+  <si>
+    <t>Варлакова Ю.Р.</t>
+  </si>
+  <si>
     <t>Алгоритмы и методы программирования, п/г 1, К503</t>
   </si>
   <si>
     <t>Алгоритмы и методы программирования, п/г 2, К503</t>
   </si>
   <si>
+    <t>Гончаров А.Р.</t>
+  </si>
+  <si>
     <t>Правоведение (лек 32 ч)</t>
   </si>
   <si>
+    <t>Ашарин А.А.</t>
+  </si>
+  <si>
+    <t>Ямпольская Н.Ю.</t>
+  </si>
+  <si>
+    <t>Варлакова Ю.Р./Попова Е.В.</t>
+  </si>
+  <si>
     <t>Основы личной и профессиональной эффективности (пр), К437</t>
   </si>
   <si>
@@ -200,18 +254,36 @@
     <t>Иностранный язык, п/г 2, К314</t>
   </si>
   <si>
+    <t>Костюнина М.В.</t>
+  </si>
+  <si>
+    <t>Подлуцкая К.А.</t>
+  </si>
+  <si>
     <t>Основы проектной деятельности (лек 16 ч)</t>
   </si>
   <si>
+    <t>Гаврилов А.С.</t>
+  </si>
+  <si>
     <t>Экономика предприятия (лек), К511</t>
   </si>
   <si>
     <t>Экономика предприятия (пр), К511</t>
   </si>
   <si>
+    <t>Макаренко И.В.</t>
+  </si>
+  <si>
     <t>Технологии программирования, п/г 1, ЭОиДОТ//</t>
   </si>
   <si>
+    <t>Осипова А.В./Курамшина А.В.</t>
+  </si>
+  <si>
+    <t>Воронина Е.В.</t>
+  </si>
+  <si>
     <t>Работа в команде (пр), К429// Учебная практика, научно-исследовательская работа (получение первичных навыков научно-исследовательской работы), К429</t>
   </si>
   <si>
@@ -242,15 +314,33 @@
     <t>Психология инклюзивного общества (лекция 16 ч)</t>
   </si>
   <si>
+    <t>Усаева Н.Р.</t>
+  </si>
+  <si>
+    <t>Батыршина К.Г.</t>
+  </si>
+  <si>
+    <t>Курц М.А.</t>
+  </si>
+  <si>
     <t>//Бизнес- планирование (лек), К511</t>
   </si>
   <si>
     <t>//Бизнес- планирование (пр), К511</t>
   </si>
   <si>
+    <t>Новичков Н.А.</t>
+  </si>
+  <si>
+    <t>Колосова О.Г.</t>
+  </si>
+  <si>
     <t>Анализ и диагностика финансово-хозяйственной деятельности корпораций (лек)/(пр), К511</t>
   </si>
   <si>
+    <t>Антонов Л.А.</t>
+  </si>
+  <si>
     <t>Экономическое обоснование цифровых решений (лек)/(пр), К511</t>
   </si>
   <si>
@@ -282,6 +372,9 @@
   </si>
   <si>
     <t>Экономическая оценка инвестиций (пр), К504//  Философия  (пр), К429</t>
+  </si>
+  <si>
+    <t>Заведеев Е.В./Калинина Е.А.</t>
   </si>
   <si>
     <t>Иностранный язык, п/г 2, К508</t>
@@ -399,7 +492,7 @@
       <charset val="204"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -418,12 +511,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="49">
+  <borders count="55">
     <border>
       <left/>
       <right/>
@@ -531,6 +630,49 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -923,6 +1065,26 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -959,6 +1121,21 @@
         <color indexed="64"/>
       </top>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1045,7 +1222,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="188">
+  <cellXfs count="207">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1088,42 +1265,48 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" textRotation="255"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1142,364 +1325,379 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="37" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="40" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Нейтральный" xfId="2" builtinId="28"/>
@@ -1829,7 +2027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="6.85546875" style="2" customWidth="1"/>
@@ -1838,10 +2036,11 @@
     <col min="4" max="4" width="18.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="20.28515625" style="2" customWidth="1"/>
     <col min="6" max="6" width="20.85546875" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="2"/>
+    <col min="7" max="7" width="18.140625" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1849,15 +2048,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -1865,39 +2064,39 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
       <c r="E4" s="5"/>
       <c r="F4" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="8" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="12" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="10">
@@ -1907,35 +2106,35 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="15" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="F7" s="16" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="75" t="s">
-        <v>43</v>
-      </c>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="75"/>
-    </row>
-    <row r="9" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+        <v>26</v>
+      </c>
+      <c r="C8" s="94" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="94"/>
+      <c r="E8" s="94"/>
+      <c r="F8" s="94"/>
+    </row>
+    <row r="9" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>0</v>
@@ -1946,340 +2145,405 @@
       <c r="D9" s="21"/>
       <c r="E9" s="22"/>
       <c r="F9" s="23"/>
-    </row>
-    <row r="10" spans="1:6" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="25">
+      <c r="G9" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="26">
         <v>2</v>
       </c>
-      <c r="C10" s="76" t="s">
-        <v>49</v>
-      </c>
-      <c r="D10" s="77"/>
-      <c r="E10" s="77"/>
-      <c r="F10" s="78"/>
-    </row>
-    <row r="11" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="26"/>
-      <c r="B11" s="27">
+      <c r="C10" s="95" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" s="96"/>
+      <c r="E10" s="96"/>
+      <c r="F10" s="97"/>
+      <c r="G10" s="53" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="28"/>
+      <c r="B11" s="29">
         <v>3</v>
       </c>
-      <c r="C11" s="71" t="s">
-        <v>48</v>
-      </c>
-      <c r="D11" s="88"/>
-      <c r="E11" s="88"/>
-      <c r="F11" s="74"/>
-    </row>
-    <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="26"/>
-      <c r="B12" s="27">
+      <c r="C11" s="107" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" s="108"/>
+      <c r="E11" s="108"/>
+      <c r="F11" s="109"/>
+      <c r="G11" s="54" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="28"/>
+      <c r="B12" s="29">
         <v>4</v>
       </c>
-      <c r="C12" s="92"/>
-      <c r="D12" s="93"/>
-      <c r="E12" s="93"/>
-      <c r="F12" s="94"/>
-    </row>
-    <row r="13" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="28"/>
-      <c r="B13" s="29">
+      <c r="C12" s="113"/>
+      <c r="D12" s="114"/>
+      <c r="E12" s="114"/>
+      <c r="F12" s="115"/>
+      <c r="G12" s="51"/>
+    </row>
+    <row r="13" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="31"/>
+      <c r="B13" s="32">
         <v>5</v>
       </c>
-      <c r="C13" s="85"/>
-      <c r="D13" s="86"/>
-      <c r="E13" s="86"/>
-      <c r="F13" s="87"/>
-    </row>
-    <row r="14" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="31">
+      <c r="C13" s="104"/>
+      <c r="D13" s="105"/>
+      <c r="E13" s="105"/>
+      <c r="F13" s="106"/>
+      <c r="G13" s="33"/>
+    </row>
+    <row r="14" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="35">
         <v>1</v>
       </c>
-      <c r="C14" s="79"/>
-      <c r="D14" s="80"/>
-      <c r="E14" s="80"/>
-      <c r="F14" s="81"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="26"/>
-      <c r="B15" s="27">
+      <c r="C14" s="98"/>
+      <c r="D14" s="99"/>
+      <c r="E14" s="99"/>
+      <c r="F14" s="100"/>
+      <c r="G14" s="53"/>
+    </row>
+    <row r="15" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="28"/>
+      <c r="B15" s="29">
         <v>2</v>
       </c>
-      <c r="C15" s="71" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="88"/>
-      <c r="E15" s="88"/>
-      <c r="F15" s="74"/>
-    </row>
-    <row r="16" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27">
+      <c r="C15" s="107" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="108"/>
+      <c r="E15" s="108"/>
+      <c r="F15" s="109"/>
+      <c r="G15" s="54" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="23.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29">
         <v>3</v>
       </c>
-      <c r="C16" s="53" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" s="54"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="55"/>
-    </row>
-    <row r="17" spans="1:6" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="32"/>
-      <c r="B17" s="29">
+      <c r="C16" s="123" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="124"/>
+      <c r="E16" s="124"/>
+      <c r="F16" s="125"/>
+      <c r="G16" s="54" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="36"/>
+      <c r="B17" s="32">
         <v>4</v>
       </c>
-      <c r="C17" s="89" t="s">
-        <v>26</v>
-      </c>
-      <c r="D17" s="90"/>
-      <c r="E17" s="90"/>
-      <c r="F17" s="91"/>
-    </row>
-    <row r="18" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="31">
+      <c r="C17" s="110" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="111"/>
+      <c r="E17" s="111"/>
+      <c r="F17" s="112"/>
+      <c r="G17" s="52" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="35">
         <v>1</v>
       </c>
-      <c r="C18" s="95"/>
-      <c r="D18" s="96"/>
-      <c r="E18" s="97" t="s">
-        <v>46</v>
-      </c>
-      <c r="F18" s="98"/>
-    </row>
-    <row r="19" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="26"/>
-      <c r="B19" s="27">
+      <c r="C18" s="116"/>
+      <c r="D18" s="117"/>
+      <c r="E18" s="118" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" s="119"/>
+      <c r="G18" s="53" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="28"/>
+      <c r="B19" s="29">
         <v>2</v>
       </c>
-      <c r="C19" s="82" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" s="83"/>
-      <c r="E19" s="83"/>
-      <c r="F19" s="84"/>
-    </row>
-    <row r="20" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27">
+      <c r="C19" s="101" t="s">
+        <v>70</v>
+      </c>
+      <c r="D19" s="102"/>
+      <c r="E19" s="102"/>
+      <c r="F19" s="103"/>
+      <c r="G19" s="54" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="28"/>
+      <c r="B20" s="29">
         <v>3</v>
       </c>
-      <c r="C20" s="56" t="s">
-        <v>45</v>
-      </c>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="58"/>
-    </row>
-    <row r="21" spans="1:6" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="32"/>
-      <c r="B21" s="29">
+      <c r="C20" s="126" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="127"/>
+      <c r="E20" s="127"/>
+      <c r="F20" s="128"/>
+      <c r="G20" s="54" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="36"/>
+      <c r="B21" s="32">
         <v>4</v>
       </c>
-      <c r="C21" s="68"/>
-      <c r="D21" s="69"/>
-      <c r="E21" s="69"/>
-      <c r="F21" s="70"/>
-    </row>
-    <row r="22" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="31">
+      <c r="C21" s="138"/>
+      <c r="D21" s="139"/>
+      <c r="E21" s="139"/>
+      <c r="F21" s="140"/>
+      <c r="G21" s="33"/>
+    </row>
+    <row r="22" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="35">
         <v>2</v>
       </c>
-      <c r="C22" s="65"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
-      <c r="F22" s="67"/>
-    </row>
-    <row r="23" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="26"/>
-      <c r="B23" s="27">
+      <c r="C22" s="135"/>
+      <c r="D22" s="136"/>
+      <c r="E22" s="136"/>
+      <c r="F22" s="137"/>
+      <c r="G22" s="27"/>
+    </row>
+    <row r="23" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="28"/>
+      <c r="B23" s="29">
         <v>3</v>
       </c>
-      <c r="C23" s="71" t="s">
+      <c r="C23" s="107" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" s="141"/>
+      <c r="E23" s="142" t="s">
+        <v>75</v>
+      </c>
+      <c r="F23" s="109"/>
+      <c r="G23" s="54" t="s">
         <v>56</v>
       </c>
-      <c r="D23" s="72"/>
-      <c r="E23" s="73" t="s">
+    </row>
+    <row r="24" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="28"/>
+      <c r="B24" s="29">
+        <v>4</v>
+      </c>
+      <c r="C24" s="123" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" s="124"/>
+      <c r="E24" s="124"/>
+      <c r="F24" s="125"/>
+      <c r="G24" s="54" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="36"/>
+      <c r="B25" s="32">
+        <v>5</v>
+      </c>
+      <c r="C25" s="132" t="s">
+        <v>73</v>
+      </c>
+      <c r="D25" s="133"/>
+      <c r="E25" s="133"/>
+      <c r="F25" s="134"/>
+      <c r="G25" s="54" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="35">
+        <v>1</v>
+      </c>
+      <c r="C26" s="129" t="s">
+        <v>120</v>
+      </c>
+      <c r="D26" s="130"/>
+      <c r="E26" s="130"/>
+      <c r="F26" s="131"/>
+      <c r="G26" s="53" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="37"/>
+      <c r="B27" s="29">
+        <v>2</v>
+      </c>
+      <c r="C27" s="123" t="s">
+        <v>71</v>
+      </c>
+      <c r="D27" s="124"/>
+      <c r="E27" s="124"/>
+      <c r="F27" s="125"/>
+      <c r="G27" s="54" t="s">
         <v>57</v>
       </c>
-      <c r="F23" s="74"/>
-    </row>
-    <row r="24" spans="1:6" ht="20.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A24" s="26"/>
-      <c r="B24" s="27">
+    </row>
+    <row r="28" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="37"/>
+      <c r="B28" s="29">
+        <v>3</v>
+      </c>
+      <c r="C28" s="120"/>
+      <c r="D28" s="121"/>
+      <c r="E28" s="121"/>
+      <c r="F28" s="122"/>
+      <c r="G28" s="54"/>
+    </row>
+    <row r="29" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="38"/>
+      <c r="B29" s="32">
         <v>4</v>
       </c>
-      <c r="C24" s="53" t="s">
-        <v>54</v>
-      </c>
-      <c r="D24" s="54"/>
-      <c r="E24" s="54"/>
-      <c r="F24" s="55"/>
-    </row>
-    <row r="25" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="32"/>
-      <c r="B25" s="29">
+      <c r="C29" s="75"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="76"/>
+      <c r="F29" s="77"/>
+      <c r="G29" s="33"/>
+    </row>
+    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="35">
+        <v>2</v>
+      </c>
+      <c r="C30" s="78" t="s">
+        <v>28</v>
+      </c>
+      <c r="D30" s="79"/>
+      <c r="E30" s="79"/>
+      <c r="F30" s="80"/>
+      <c r="G30" s="53" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="37"/>
+      <c r="B31" s="29">
+        <v>4</v>
+      </c>
+      <c r="C31" s="91"/>
+      <c r="D31" s="92"/>
+      <c r="E31" s="92"/>
+      <c r="F31" s="93"/>
+      <c r="G31" s="30"/>
+    </row>
+    <row r="32" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="40"/>
+      <c r="B32" s="29">
         <v>5</v>
       </c>
-      <c r="C25" s="62" t="s">
+      <c r="C32" s="85"/>
+      <c r="D32" s="86"/>
+      <c r="E32" s="86"/>
+      <c r="F32" s="87"/>
+      <c r="G32" s="54"/>
+    </row>
+    <row r="33" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="41"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="69"/>
+      <c r="D33" s="70"/>
+      <c r="E33" s="70"/>
+      <c r="F33" s="71"/>
+      <c r="G33" s="33"/>
+    </row>
+    <row r="34" spans="1:7" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="42"/>
+      <c r="B34" s="43"/>
+      <c r="C34" s="81"/>
+      <c r="D34" s="81"/>
+      <c r="E34" s="81"/>
+      <c r="F34" s="81"/>
+      <c r="G34" s="44"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A35" s="55"/>
+      <c r="B35" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="88" t="s">
+        <v>62</v>
+      </c>
+      <c r="D35" s="89"/>
+      <c r="E35" s="89"/>
+      <c r="F35" s="90"/>
+      <c r="G35" s="53" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A36" s="37"/>
+      <c r="B36" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="82" t="s">
+        <v>38</v>
+      </c>
+      <c r="D36" s="83"/>
+      <c r="E36" s="83"/>
+      <c r="F36" s="84"/>
+      <c r="G36" s="54" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="41"/>
+      <c r="B37" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="72" t="s">
+        <v>37</v>
+      </c>
+      <c r="D37" s="73"/>
+      <c r="E37" s="73"/>
+      <c r="F37" s="74"/>
+      <c r="G37" s="52" t="s">
         <v>55</v>
       </c>
-      <c r="D25" s="63"/>
-      <c r="E25" s="63"/>
-      <c r="F25" s="64"/>
-    </row>
-    <row r="26" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="31">
-        <v>1</v>
-      </c>
-      <c r="C26" s="59" t="s">
-        <v>89</v>
-      </c>
-      <c r="D26" s="60"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="61"/>
-    </row>
-    <row r="27" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="33"/>
-      <c r="B27" s="27">
-        <v>2</v>
-      </c>
-      <c r="C27" s="53" t="s">
-        <v>53</v>
-      </c>
-      <c r="D27" s="54"/>
-      <c r="E27" s="54"/>
-      <c r="F27" s="55"/>
-    </row>
-    <row r="28" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="33"/>
-      <c r="B28" s="27">
-        <v>3</v>
-      </c>
-      <c r="C28" s="50"/>
-      <c r="D28" s="51"/>
-      <c r="E28" s="51"/>
-      <c r="F28" s="52"/>
-    </row>
-    <row r="29" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="34"/>
-      <c r="B29" s="29">
-        <v>4</v>
-      </c>
-      <c r="C29" s="105"/>
-      <c r="D29" s="106"/>
-      <c r="E29" s="106"/>
-      <c r="F29" s="107"/>
-    </row>
-    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="35" t="s">
-        <v>24</v>
-      </c>
-      <c r="B30" s="31">
-        <v>2</v>
-      </c>
-      <c r="C30" s="108" t="s">
-        <v>27</v>
-      </c>
-      <c r="D30" s="109"/>
-      <c r="E30" s="109"/>
-      <c r="F30" s="110"/>
-    </row>
-    <row r="31" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="33"/>
-      <c r="B31" s="27">
-        <v>4</v>
-      </c>
-      <c r="C31" s="121"/>
-      <c r="D31" s="122"/>
-      <c r="E31" s="122"/>
-      <c r="F31" s="123"/>
-    </row>
-    <row r="32" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="36"/>
-      <c r="B32" s="27">
-        <v>5</v>
-      </c>
-      <c r="C32" s="115"/>
-      <c r="D32" s="116"/>
-      <c r="E32" s="116"/>
-      <c r="F32" s="117"/>
-    </row>
-    <row r="33" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="37"/>
-      <c r="B33" s="29"/>
-      <c r="C33" s="99"/>
-      <c r="D33" s="100"/>
-      <c r="E33" s="100"/>
-      <c r="F33" s="101"/>
-    </row>
-    <row r="34" spans="1:6" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="38"/>
-      <c r="B34" s="39"/>
-      <c r="C34" s="111"/>
-      <c r="D34" s="111"/>
-      <c r="E34" s="111"/>
-      <c r="F34" s="111"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A35" s="45"/>
-      <c r="B35" s="31" t="s">
-        <v>29</v>
-      </c>
-      <c r="C35" s="118" t="s">
-        <v>47</v>
-      </c>
-      <c r="D35" s="119"/>
-      <c r="E35" s="119"/>
-      <c r="F35" s="120"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A36" s="33"/>
-      <c r="B36" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="C36" s="112" t="s">
-        <v>34</v>
-      </c>
-      <c r="D36" s="113"/>
-      <c r="E36" s="113"/>
-      <c r="F36" s="114"/>
-    </row>
-    <row r="37" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="37"/>
-      <c r="B37" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37" s="102" t="s">
-        <v>33</v>
-      </c>
-      <c r="D37" s="103"/>
-      <c r="E37" s="103"/>
-      <c r="F37" s="104"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A39" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A40" s="2" t="s">
         <v>14</v>
       </c>
@@ -2289,26 +2553,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="C13:F13"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="E18:F18"/>
     <mergeCell ref="C28:F28"/>
     <mergeCell ref="C27:F27"/>
     <mergeCell ref="C20:D20"/>
@@ -2321,6 +2565,26 @@
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="C24:F24"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C31:F31"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" sqref="C6"/>
@@ -2351,7 +2615,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
@@ -2360,9 +2624,10 @@
     <col min="4" max="4" width="17.5703125" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="19.140625" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -2373,10 +2638,11 @@
       <c r="F1" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G1" s="2"/>
+    </row>
+    <row r="2" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2385,8 +2651,9 @@
       <c r="F2" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -2397,42 +2664,45 @@
       <c r="F3" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
       <c r="E4" s="5"/>
       <c r="F4" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+        <v>50</v>
+      </c>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A5" s="8" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="9" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A6" s="12" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="10">
@@ -2441,38 +2711,41 @@
       <c r="F6" s="11" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A7" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="14" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="15" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F7" s="16" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" spans="1:7" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="75" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="75"/>
-    </row>
-    <row r="9" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="C8" s="94" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="94"/>
+      <c r="E8" s="94"/>
+      <c r="F8" s="94"/>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>0</v>
@@ -2483,352 +2756,417 @@
       <c r="D9" s="21"/>
       <c r="E9" s="22"/>
       <c r="F9" s="23"/>
-    </row>
-    <row r="10" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A10" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="25">
+      <c r="G9" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A10" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="26">
         <v>1</v>
       </c>
-      <c r="C10" s="108" t="s">
+      <c r="C10" s="78" t="s">
+        <v>114</v>
+      </c>
+      <c r="D10" s="79"/>
+      <c r="E10" s="79"/>
+      <c r="F10" s="80"/>
+      <c r="G10" s="53" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A11" s="28"/>
+      <c r="B11" s="29">
+        <v>2</v>
+      </c>
+      <c r="C11" s="91"/>
+      <c r="D11" s="92"/>
+      <c r="E11" s="83" t="s">
+        <v>117</v>
+      </c>
+      <c r="F11" s="84"/>
+      <c r="G11" s="54" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A12" s="28"/>
+      <c r="B12" s="29">
+        <v>3</v>
+      </c>
+      <c r="C12" s="149" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="150"/>
+      <c r="E12" s="150"/>
+      <c r="F12" s="151"/>
+      <c r="G12" s="30"/>
+    </row>
+    <row r="13" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="31"/>
+      <c r="B13" s="32">
+        <v>4</v>
+      </c>
+      <c r="C13" s="152"/>
+      <c r="D13" s="153"/>
+      <c r="E13" s="153"/>
+      <c r="F13" s="154"/>
+      <c r="G13" s="33"/>
+    </row>
+    <row r="14" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A14" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="35">
+        <v>1</v>
+      </c>
+      <c r="C14" s="155" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="156"/>
+      <c r="E14" s="156"/>
+      <c r="F14" s="157"/>
+      <c r="G14" s="53" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="28"/>
+      <c r="B15" s="29">
+        <v>2</v>
+      </c>
+      <c r="C15" s="126" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="127"/>
+      <c r="E15" s="127"/>
+      <c r="F15" s="128"/>
+      <c r="G15" s="54" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29">
+        <v>3</v>
+      </c>
+      <c r="C16" s="123"/>
+      <c r="D16" s="124"/>
+      <c r="E16" s="124"/>
+      <c r="F16" s="125"/>
+      <c r="G16" s="54"/>
+    </row>
+    <row r="17" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="36"/>
+      <c r="B17" s="32">
+        <v>4</v>
+      </c>
+      <c r="C17" s="138"/>
+      <c r="D17" s="139"/>
+      <c r="E17" s="139"/>
+      <c r="F17" s="140"/>
+      <c r="G17" s="33"/>
+    </row>
+    <row r="18" spans="1:7" ht="56.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="35">
+        <v>1</v>
+      </c>
+      <c r="C18" s="146" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="147"/>
+      <c r="E18" s="147"/>
+      <c r="F18" s="148"/>
+      <c r="G18" s="54" t="s">
         <v>84</v>
       </c>
-      <c r="D10" s="109"/>
-      <c r="E10" s="109"/>
-      <c r="F10" s="110"/>
-    </row>
-    <row r="11" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A11" s="26"/>
-      <c r="B11" s="27">
+    </row>
+    <row r="19" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="28"/>
+      <c r="B19" s="29">
         <v>2</v>
       </c>
-      <c r="C11" s="121"/>
-      <c r="D11" s="122"/>
-      <c r="E11" s="113" t="s">
-        <v>86</v>
-      </c>
-      <c r="F11" s="114"/>
-    </row>
-    <row r="12" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A12" s="26"/>
-      <c r="B12" s="27">
+      <c r="C19" s="123" t="s">
+        <v>87</v>
+      </c>
+      <c r="D19" s="124"/>
+      <c r="E19" s="124"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="54" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A20" s="28"/>
+      <c r="B20" s="29">
         <v>3</v>
       </c>
-      <c r="C12" s="151" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="152"/>
-      <c r="E12" s="152"/>
-      <c r="F12" s="153"/>
-    </row>
-    <row r="13" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="28"/>
-      <c r="B13" s="29">
+      <c r="C20" s="143" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" s="144"/>
+      <c r="E20" s="144"/>
+      <c r="F20" s="145"/>
+      <c r="G20" s="54" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="36"/>
+      <c r="B21" s="32">
         <v>4</v>
       </c>
-      <c r="C13" s="154"/>
-      <c r="D13" s="155"/>
-      <c r="E13" s="155"/>
-      <c r="F13" s="156"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A14" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="31">
+      <c r="C21" s="158"/>
+      <c r="D21" s="159"/>
+      <c r="E21" s="159"/>
+      <c r="F21" s="160"/>
+      <c r="G21" s="33"/>
+    </row>
+    <row r="22" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A22" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="35">
         <v>1</v>
       </c>
-      <c r="C14" s="157" t="s">
-        <v>59</v>
-      </c>
-      <c r="D14" s="158"/>
-      <c r="E14" s="158"/>
-      <c r="F14" s="159"/>
-    </row>
-    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="26"/>
-      <c r="B15" s="27">
+      <c r="C22" s="170" t="s">
+        <v>113</v>
+      </c>
+      <c r="D22" s="171"/>
+      <c r="E22" s="172"/>
+      <c r="F22" s="173"/>
+      <c r="G22" s="65" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A23" s="28"/>
+      <c r="B23" s="29">
         <v>2</v>
       </c>
-      <c r="C15" s="56" t="s">
-        <v>60</v>
-      </c>
-      <c r="D15" s="57"/>
-      <c r="E15" s="57"/>
-      <c r="F15" s="58"/>
-    </row>
-    <row r="16" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27">
+      <c r="C23" s="91"/>
+      <c r="D23" s="92"/>
+      <c r="E23" s="92"/>
+      <c r="F23" s="93"/>
+      <c r="G23" s="30"/>
+    </row>
+    <row r="24" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A24" s="28"/>
+      <c r="B24" s="29">
         <v>3</v>
       </c>
-      <c r="C16" s="53"/>
-      <c r="D16" s="54"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="55"/>
-    </row>
-    <row r="17" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="32"/>
-      <c r="B17" s="29">
+      <c r="C24" s="161" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="162"/>
+      <c r="E24" s="162"/>
+      <c r="F24" s="163"/>
+      <c r="G24" s="47"/>
+    </row>
+    <row r="25" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="36"/>
+      <c r="B25" s="32">
         <v>4</v>
       </c>
-      <c r="C17" s="68"/>
-      <c r="D17" s="69"/>
-      <c r="E17" s="69"/>
-      <c r="F17" s="70"/>
-    </row>
-    <row r="18" spans="1:6" ht="56.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="31">
-        <v>1</v>
-      </c>
-      <c r="C18" s="163" t="s">
-        <v>62</v>
-      </c>
-      <c r="D18" s="164"/>
-      <c r="E18" s="164"/>
-      <c r="F18" s="165"/>
-    </row>
-    <row r="19" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="26"/>
-      <c r="B19" s="27">
+      <c r="C25" s="164"/>
+      <c r="D25" s="165"/>
+      <c r="E25" s="165"/>
+      <c r="F25" s="166"/>
+      <c r="G25" s="30"/>
+    </row>
+    <row r="26" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A26" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="35">
+        <v>3</v>
+      </c>
+      <c r="C26" s="78" t="s">
+        <v>88</v>
+      </c>
+      <c r="D26" s="79"/>
+      <c r="E26" s="79"/>
+      <c r="F26" s="80"/>
+      <c r="G26" s="66" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A27" s="37"/>
+      <c r="B27" s="29">
+        <v>4</v>
+      </c>
+      <c r="C27" s="126" t="s">
+        <v>89</v>
+      </c>
+      <c r="D27" s="127"/>
+      <c r="E27" s="127"/>
+      <c r="F27" s="128"/>
+      <c r="G27" s="67" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="37"/>
+      <c r="B28" s="29">
+        <v>7</v>
+      </c>
+      <c r="C28" s="126" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" s="127"/>
+      <c r="E28" s="127"/>
+      <c r="F28" s="128"/>
+      <c r="G28" s="54" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="38"/>
+      <c r="B29" s="32">
+        <v>8</v>
+      </c>
+      <c r="C29" s="174" t="s">
+        <v>83</v>
+      </c>
+      <c r="D29" s="175"/>
+      <c r="E29" s="176"/>
+      <c r="F29" s="177"/>
+      <c r="G29" s="52" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A30" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="35">
         <v>2</v>
       </c>
-      <c r="C19" s="53" t="s">
-        <v>63</v>
-      </c>
-      <c r="D19" s="54"/>
-      <c r="E19" s="54"/>
-      <c r="F19" s="55"/>
-    </row>
-    <row r="20" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27">
+      <c r="C30" s="167"/>
+      <c r="D30" s="168"/>
+      <c r="E30" s="168"/>
+      <c r="F30" s="169"/>
+      <c r="G30" s="53"/>
+    </row>
+    <row r="31" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="37"/>
+      <c r="B31" s="29">
         <v>3</v>
       </c>
-      <c r="C20" s="160" t="s">
-        <v>85</v>
-      </c>
-      <c r="D20" s="161"/>
-      <c r="E20" s="161"/>
-      <c r="F20" s="162"/>
-    </row>
-    <row r="21" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="32"/>
-      <c r="B21" s="29">
+      <c r="C31" s="107"/>
+      <c r="D31" s="108"/>
+      <c r="E31" s="108"/>
+      <c r="F31" s="109"/>
+      <c r="G31" s="54"/>
+    </row>
+    <row r="32" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A32" s="40"/>
+      <c r="B32" s="29">
         <v>4</v>
       </c>
-      <c r="C21" s="131"/>
-      <c r="D21" s="132"/>
-      <c r="E21" s="132"/>
-      <c r="F21" s="133"/>
-    </row>
-    <row r="22" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A22" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="31">
-        <v>1</v>
-      </c>
-      <c r="C22" s="143" t="s">
-        <v>83</v>
-      </c>
-      <c r="D22" s="144"/>
-      <c r="E22" s="145"/>
-      <c r="F22" s="146"/>
-    </row>
-    <row r="23" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A23" s="26"/>
-      <c r="B23" s="27">
-        <v>2</v>
-      </c>
-      <c r="C23" s="121"/>
-      <c r="D23" s="122"/>
-      <c r="E23" s="122"/>
-      <c r="F23" s="123"/>
-    </row>
-    <row r="24" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A24" s="26"/>
-      <c r="B24" s="27">
-        <v>3</v>
-      </c>
-      <c r="C24" s="134" t="s">
-        <v>27</v>
-      </c>
-      <c r="D24" s="135"/>
-      <c r="E24" s="135"/>
-      <c r="F24" s="136"/>
-    </row>
-    <row r="25" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="32"/>
-      <c r="B25" s="29">
-        <v>4</v>
-      </c>
-      <c r="C25" s="137"/>
-      <c r="D25" s="138"/>
-      <c r="E25" s="138"/>
-      <c r="F25" s="139"/>
-    </row>
-    <row r="26" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A26" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="31">
-        <v>3</v>
-      </c>
-      <c r="C26" s="108" t="s">
-        <v>64</v>
-      </c>
-      <c r="D26" s="109"/>
-      <c r="E26" s="109"/>
-      <c r="F26" s="110"/>
-    </row>
-    <row r="27" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A27" s="33"/>
-      <c r="B27" s="27">
-        <v>4</v>
-      </c>
-      <c r="C27" s="56" t="s">
-        <v>65</v>
-      </c>
-      <c r="D27" s="57"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="58"/>
-    </row>
-    <row r="28" spans="1:6" ht="37.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="33"/>
-      <c r="B28" s="27">
-        <v>7</v>
-      </c>
-      <c r="C28" s="56" t="s">
-        <v>87</v>
-      </c>
-      <c r="D28" s="57"/>
-      <c r="E28" s="57"/>
-      <c r="F28" s="58"/>
-    </row>
-    <row r="29" spans="1:6" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="34"/>
-      <c r="B29" s="29">
-        <v>8</v>
-      </c>
-      <c r="C29" s="147" t="s">
-        <v>61</v>
-      </c>
-      <c r="D29" s="148"/>
-      <c r="E29" s="149"/>
-      <c r="F29" s="150"/>
-    </row>
-    <row r="30" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A30" s="35" t="s">
-        <v>24</v>
-      </c>
-      <c r="B30" s="31">
-        <v>2</v>
-      </c>
-      <c r="C30" s="140"/>
-      <c r="D30" s="141"/>
-      <c r="E30" s="141"/>
-      <c r="F30" s="142"/>
-    </row>
-    <row r="31" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="33"/>
-      <c r="B31" s="27">
-        <v>3</v>
-      </c>
-      <c r="C31" s="71"/>
-      <c r="D31" s="88"/>
-      <c r="E31" s="88"/>
-      <c r="F31" s="74"/>
-    </row>
-    <row r="32" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A32" s="36"/>
-      <c r="B32" s="27">
-        <v>4</v>
-      </c>
-      <c r="C32" s="53" t="s">
-        <v>66</v>
-      </c>
-      <c r="D32" s="54"/>
-      <c r="E32" s="54"/>
-      <c r="F32" s="55"/>
-    </row>
-    <row r="33" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="37"/>
-      <c r="B33" s="29"/>
-      <c r="C33" s="99"/>
-      <c r="D33" s="100"/>
-      <c r="E33" s="100"/>
-      <c r="F33" s="101"/>
-    </row>
-    <row r="34" spans="1:6" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="38"/>
-      <c r="B34" s="39"/>
-      <c r="C34" s="124"/>
-      <c r="D34" s="124"/>
-      <c r="E34" s="124"/>
-      <c r="F34" s="124"/>
-    </row>
-    <row r="35" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A35" s="40"/>
-      <c r="B35" s="42" t="s">
-        <v>29</v>
-      </c>
-      <c r="C35" s="125" t="s">
-        <v>36</v>
-      </c>
-      <c r="D35" s="126"/>
-      <c r="E35" s="126"/>
-      <c r="F35" s="127"/>
-    </row>
-    <row r="36" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A36" s="41"/>
-      <c r="B36" s="44" t="s">
-        <v>29</v>
-      </c>
-      <c r="C36" s="128" t="s">
-        <v>58</v>
-      </c>
-      <c r="D36" s="129"/>
-      <c r="E36" s="129"/>
-      <c r="F36" s="130"/>
-    </row>
-    <row r="37" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A37" s="37"/>
-      <c r="B37" s="43" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37" s="102" t="s">
-        <v>37</v>
-      </c>
-      <c r="D37" s="103"/>
-      <c r="E37" s="103"/>
-      <c r="F37" s="104"/>
-    </row>
-    <row r="38" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="C32" s="123" t="s">
+        <v>90</v>
+      </c>
+      <c r="D32" s="124"/>
+      <c r="E32" s="124"/>
+      <c r="F32" s="125"/>
+      <c r="G32" s="54" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="41"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="69"/>
+      <c r="D33" s="70"/>
+      <c r="E33" s="70"/>
+      <c r="F33" s="71"/>
+      <c r="G33" s="52"/>
+    </row>
+    <row r="34" spans="1:7" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="42"/>
+      <c r="B34" s="43"/>
+      <c r="C34" s="178"/>
+      <c r="D34" s="178"/>
+      <c r="E34" s="178"/>
+      <c r="F34" s="178"/>
+      <c r="G34" s="44"/>
+    </row>
+    <row r="35" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A35" s="45"/>
+      <c r="B35" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="179" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35" s="180"/>
+      <c r="E35" s="180"/>
+      <c r="F35" s="181"/>
+      <c r="G35" s="57" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A36" s="46"/>
+      <c r="B36" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="182" t="s">
+        <v>78</v>
+      </c>
+      <c r="D36" s="183"/>
+      <c r="E36" s="183"/>
+      <c r="F36" s="184"/>
+      <c r="G36" s="58" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="41"/>
+      <c r="B37" s="49" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="72" t="s">
+        <v>42</v>
+      </c>
+      <c r="D37" s="73"/>
+      <c r="E37" s="73"/>
+      <c r="F37" s="74"/>
+      <c r="G37" s="56" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
-    </row>
-    <row r="39" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G38" s="2"/>
+    </row>
+    <row r="39" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A39" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
-    </row>
-    <row r="40" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G39" s="2"/>
+    </row>
+    <row r="40" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A40" s="2" t="s">
         <v>14</v>
       </c>
@@ -2839,9 +3177,27 @@
       </c>
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="E29:F29"/>
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="C33:F33"/>
     <mergeCell ref="C8:F8"/>
@@ -2857,23 +3213,6 @@
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="C32:F32"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E5">
@@ -2904,7 +3243,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
@@ -2913,9 +3252,10 @@
     <col min="4" max="4" width="18.140625" customWidth="1"/>
     <col min="5" max="5" width="18.5703125" customWidth="1"/>
     <col min="6" max="6" width="19.42578125" customWidth="1"/>
+    <col min="7" max="7" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -2926,10 +3266,11 @@
       <c r="F1" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G1" s="2"/>
+    </row>
+    <row r="2" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2938,8 +3279,9 @@
       <c r="F2" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -2950,42 +3292,45 @@
       <c r="F3" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A4" s="4" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
       <c r="E4" s="5"/>
       <c r="F4" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+        <v>50</v>
+      </c>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A5" s="8" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="9" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A6" s="12" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="10">
@@ -2994,38 +3339,41 @@
       <c r="F6" s="11" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A7" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="14" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D7" s="14"/>
       <c r="E7" s="15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F7" s="16" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" spans="1:7" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="75" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="75"/>
-    </row>
-    <row r="9" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="C8" s="94" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="94"/>
+      <c r="E8" s="94"/>
+      <c r="F8" s="94"/>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A9" s="18" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="19" t="s">
         <v>0</v>
@@ -3036,330 +3384,387 @@
       <c r="D9" s="21"/>
       <c r="E9" s="22"/>
       <c r="F9" s="23"/>
-    </row>
-    <row r="10" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A10" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="25">
+      <c r="G9" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A10" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="26">
         <v>1</v>
       </c>
-      <c r="C10" s="166"/>
-      <c r="D10" s="167"/>
-      <c r="E10" s="167"/>
-      <c r="F10" s="168"/>
-    </row>
-    <row r="11" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A11" s="26"/>
-      <c r="B11" s="27">
+      <c r="C10" s="195"/>
+      <c r="D10" s="196"/>
+      <c r="E10" s="196"/>
+      <c r="F10" s="197"/>
+      <c r="G10" s="53"/>
+    </row>
+    <row r="11" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A11" s="28"/>
+      <c r="B11" s="29">
         <v>2</v>
       </c>
-      <c r="C11" s="160" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" s="161"/>
-      <c r="E11" s="161"/>
-      <c r="F11" s="162"/>
-    </row>
-    <row r="12" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A12" s="26"/>
-      <c r="B12" s="27">
+      <c r="C11" s="143" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="144"/>
+      <c r="E11" s="144"/>
+      <c r="F11" s="145"/>
+      <c r="G11" s="54" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A12" s="28"/>
+      <c r="B12" s="29">
         <v>3</v>
       </c>
-      <c r="C12" s="134" t="s">
-        <v>76</v>
-      </c>
-      <c r="D12" s="135"/>
-      <c r="E12" s="135"/>
-      <c r="F12" s="136"/>
-    </row>
-    <row r="13" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="28"/>
-      <c r="B13" s="29">
+      <c r="C12" s="161" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" s="162"/>
+      <c r="E12" s="162"/>
+      <c r="F12" s="163"/>
+      <c r="G12" s="54" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="31"/>
+      <c r="B13" s="32">
         <v>4</v>
       </c>
-      <c r="C13" s="85"/>
-      <c r="D13" s="86"/>
-      <c r="E13" s="86"/>
-      <c r="F13" s="87"/>
-    </row>
-    <row r="14" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A14" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="31" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" s="169" t="s">
-        <v>68</v>
-      </c>
-      <c r="D14" s="97"/>
-      <c r="E14" s="97"/>
-      <c r="F14" s="98"/>
-    </row>
-    <row r="15" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="26"/>
-      <c r="B15" s="27">
+      <c r="C13" s="104"/>
+      <c r="D13" s="105"/>
+      <c r="E13" s="105"/>
+      <c r="F13" s="106"/>
+      <c r="G13" s="33"/>
+    </row>
+    <row r="14" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A14" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="198" t="s">
+        <v>92</v>
+      </c>
+      <c r="D14" s="118"/>
+      <c r="E14" s="118"/>
+      <c r="F14" s="119"/>
+      <c r="G14" s="27"/>
+    </row>
+    <row r="15" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="28"/>
+      <c r="B15" s="29">
         <v>4</v>
       </c>
-      <c r="C15" s="82" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" s="83"/>
-      <c r="E15" s="83"/>
-      <c r="F15" s="84"/>
-    </row>
-    <row r="16" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27">
+      <c r="C15" s="101" t="s">
+        <v>103</v>
+      </c>
+      <c r="D15" s="102"/>
+      <c r="E15" s="102"/>
+      <c r="F15" s="103"/>
+      <c r="G15" s="54" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="17.25" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="28"/>
+      <c r="B16" s="29">
         <v>5</v>
       </c>
-      <c r="C16" s="53" t="s">
-        <v>88</v>
-      </c>
-      <c r="D16" s="54"/>
-      <c r="E16" s="54"/>
-      <c r="F16" s="55"/>
-    </row>
-    <row r="17" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="32"/>
-      <c r="B17" s="29">
+      <c r="C16" s="123" t="s">
+        <v>119</v>
+      </c>
+      <c r="D16" s="124"/>
+      <c r="E16" s="124"/>
+      <c r="F16" s="125"/>
+      <c r="G16" s="68" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="36"/>
+      <c r="B17" s="32">
         <v>6</v>
       </c>
-      <c r="C17" s="68"/>
-      <c r="D17" s="69"/>
-      <c r="E17" s="69"/>
-      <c r="F17" s="70"/>
-    </row>
-    <row r="18" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A18" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18" s="31">
+      <c r="C17" s="138"/>
+      <c r="D17" s="139"/>
+      <c r="E17" s="139"/>
+      <c r="F17" s="140"/>
+      <c r="G17" s="33"/>
+    </row>
+    <row r="18" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A18" s="34" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="35">
         <v>1</v>
       </c>
-      <c r="C18" s="143" t="s">
-        <v>73</v>
-      </c>
-      <c r="D18" s="170"/>
-      <c r="E18" s="170"/>
-      <c r="F18" s="171"/>
-    </row>
-    <row r="19" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="26"/>
-      <c r="B19" s="27">
+      <c r="C18" s="170" t="s">
+        <v>100</v>
+      </c>
+      <c r="D18" s="199"/>
+      <c r="E18" s="199"/>
+      <c r="F18" s="200"/>
+      <c r="G18" s="57" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="28"/>
+      <c r="B19" s="29">
         <v>2</v>
       </c>
-      <c r="C19" s="53" t="s">
-        <v>75</v>
-      </c>
-      <c r="D19" s="54"/>
-      <c r="E19" s="54"/>
-      <c r="F19" s="55"/>
-    </row>
-    <row r="20" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A20" s="26"/>
-      <c r="B20" s="27">
+      <c r="C19" s="123" t="s">
+        <v>105</v>
+      </c>
+      <c r="D19" s="124"/>
+      <c r="E19" s="124"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="54" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A20" s="28"/>
+      <c r="B20" s="29">
         <v>3</v>
       </c>
-      <c r="C20" s="53" t="s">
-        <v>77</v>
-      </c>
-      <c r="D20" s="54"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="55"/>
-    </row>
-    <row r="21" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="32"/>
-      <c r="B21" s="29">
+      <c r="C20" s="123" t="s">
+        <v>107</v>
+      </c>
+      <c r="D20" s="124"/>
+      <c r="E20" s="124"/>
+      <c r="F20" s="125"/>
+      <c r="G20" s="54" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="36"/>
+      <c r="B21" s="32">
         <v>4</v>
       </c>
-      <c r="C21" s="131"/>
-      <c r="D21" s="132"/>
-      <c r="E21" s="132"/>
-      <c r="F21" s="133"/>
-    </row>
-    <row r="22" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A22" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="31">
+      <c r="C21" s="158"/>
+      <c r="D21" s="159"/>
+      <c r="E21" s="159"/>
+      <c r="F21" s="160"/>
+      <c r="G21" s="33"/>
+    </row>
+    <row r="22" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A22" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B22" s="35">
         <v>2</v>
       </c>
-      <c r="C22" s="178"/>
-      <c r="D22" s="179"/>
-      <c r="E22" s="179"/>
-      <c r="F22" s="180"/>
-    </row>
-    <row r="23" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A23" s="26"/>
-      <c r="B23" s="27">
+      <c r="C22" s="189"/>
+      <c r="D22" s="190"/>
+      <c r="E22" s="190"/>
+      <c r="F22" s="191"/>
+      <c r="G22" s="27"/>
+    </row>
+    <row r="23" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A23" s="28"/>
+      <c r="B23" s="29">
         <v>3</v>
       </c>
-      <c r="C23" s="112" t="s">
-        <v>78</v>
-      </c>
-      <c r="D23" s="113"/>
-      <c r="E23" s="113"/>
-      <c r="F23" s="114"/>
-    </row>
-    <row r="24" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A24" s="26"/>
-      <c r="B24" s="27">
+      <c r="C23" s="82" t="s">
+        <v>108</v>
+      </c>
+      <c r="D23" s="83"/>
+      <c r="E23" s="83"/>
+      <c r="F23" s="84"/>
+      <c r="G23" s="54" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A24" s="28"/>
+      <c r="B24" s="29">
         <v>4</v>
       </c>
-      <c r="C24" s="134" t="s">
-        <v>79</v>
-      </c>
-      <c r="D24" s="135"/>
-      <c r="E24" s="135"/>
-      <c r="F24" s="136"/>
-    </row>
-    <row r="25" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="32"/>
-      <c r="B25" s="29">
+      <c r="C24" s="161" t="s">
+        <v>109</v>
+      </c>
+      <c r="D24" s="162"/>
+      <c r="E24" s="162"/>
+      <c r="F24" s="163"/>
+      <c r="G24" s="64" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A25" s="36"/>
+      <c r="B25" s="32">
         <v>5</v>
       </c>
-      <c r="C25" s="181"/>
-      <c r="D25" s="182"/>
-      <c r="E25" s="182"/>
-      <c r="F25" s="183"/>
-    </row>
-    <row r="26" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A26" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="B26" s="31">
+      <c r="C25" s="192"/>
+      <c r="D25" s="193"/>
+      <c r="E25" s="193"/>
+      <c r="F25" s="194"/>
+      <c r="G25" s="54"/>
+    </row>
+    <row r="26" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A26" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="35">
         <v>1</v>
       </c>
-      <c r="C26" s="172" t="s">
-        <v>35</v>
-      </c>
-      <c r="D26" s="173"/>
-      <c r="E26" s="173"/>
-      <c r="F26" s="174"/>
-    </row>
-    <row r="27" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A27" s="33"/>
-      <c r="B27" s="27">
+      <c r="C26" s="201" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="202"/>
+      <c r="E26" s="202"/>
+      <c r="F26" s="203"/>
+      <c r="G26" s="27"/>
+    </row>
+    <row r="27" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A27" s="37"/>
+      <c r="B27" s="29">
         <v>2</v>
       </c>
-      <c r="C27" s="50"/>
-      <c r="D27" s="51"/>
-      <c r="E27" s="51"/>
-      <c r="F27" s="52"/>
-    </row>
-    <row r="28" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A28" s="33"/>
-      <c r="B28" s="27">
+      <c r="C27" s="120"/>
+      <c r="D27" s="121"/>
+      <c r="E27" s="121"/>
+      <c r="F27" s="122"/>
+      <c r="G27" s="30"/>
+    </row>
+    <row r="28" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A28" s="37"/>
+      <c r="B28" s="29">
         <v>3</v>
       </c>
-      <c r="C28" s="175"/>
-      <c r="D28" s="176"/>
-      <c r="E28" s="176"/>
-      <c r="F28" s="177"/>
-    </row>
-    <row r="29" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="34"/>
-      <c r="B29" s="29">
+      <c r="C28" s="204"/>
+      <c r="D28" s="205"/>
+      <c r="E28" s="205"/>
+      <c r="F28" s="206"/>
+      <c r="G28" s="30"/>
+    </row>
+    <row r="29" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A29" s="38"/>
+      <c r="B29" s="32">
         <v>4</v>
       </c>
-      <c r="C29" s="105"/>
-      <c r="D29" s="106"/>
-      <c r="E29" s="106"/>
-      <c r="F29" s="107"/>
-    </row>
-    <row r="30" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A30" s="35" t="s">
-        <v>24</v>
-      </c>
-      <c r="B30" s="31">
+      <c r="C29" s="75"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="76"/>
+      <c r="F29" s="77"/>
+      <c r="G29" s="33"/>
+    </row>
+    <row r="30" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A30" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="35">
         <v>2</v>
       </c>
-      <c r="C30" s="108" t="s">
-        <v>80</v>
-      </c>
-      <c r="D30" s="109"/>
-      <c r="E30" s="109"/>
-      <c r="F30" s="110"/>
-    </row>
-    <row r="31" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
-      <c r="A31" s="33"/>
-      <c r="B31" s="27">
+      <c r="C30" s="78" t="s">
+        <v>110</v>
+      </c>
+      <c r="D30" s="79"/>
+      <c r="E30" s="79"/>
+      <c r="F30" s="80"/>
+      <c r="G30" s="53" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="A31" s="37"/>
+      <c r="B31" s="29">
         <v>3</v>
       </c>
-      <c r="C31" s="112" t="s">
-        <v>81</v>
-      </c>
-      <c r="D31" s="113"/>
-      <c r="E31" s="113"/>
-      <c r="F31" s="114"/>
-    </row>
-    <row r="32" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="36"/>
-      <c r="B32" s="27">
+      <c r="C31" s="82" t="s">
+        <v>111</v>
+      </c>
+      <c r="D31" s="83"/>
+      <c r="E31" s="83"/>
+      <c r="F31" s="84"/>
+      <c r="G31" s="54" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="40"/>
+      <c r="B32" s="29">
         <v>4</v>
       </c>
-      <c r="C32" s="53" t="s">
-        <v>82</v>
-      </c>
-      <c r="D32" s="54"/>
-      <c r="E32" s="54"/>
-      <c r="F32" s="55"/>
-    </row>
-    <row r="33" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="37"/>
-      <c r="B33" s="29"/>
-      <c r="C33" s="99"/>
-      <c r="D33" s="100"/>
-      <c r="E33" s="100"/>
-      <c r="F33" s="101"/>
-    </row>
-    <row r="34" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A34" s="38"/>
-      <c r="B34" s="39"/>
-      <c r="C34" s="124"/>
-      <c r="D34" s="124"/>
-      <c r="E34" s="124"/>
-      <c r="F34" s="124"/>
-    </row>
-    <row r="35" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A35" s="49"/>
-      <c r="B35" s="48" t="s">
-        <v>29</v>
-      </c>
-      <c r="C35" s="185" t="s">
-        <v>71</v>
-      </c>
-      <c r="D35" s="186"/>
-      <c r="E35" s="186"/>
-      <c r="F35" s="187"/>
-    </row>
-    <row r="36" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="46" t="s">
-        <v>69</v>
-      </c>
-      <c r="B36" s="47"/>
-      <c r="C36" s="184" t="s">
-        <v>70</v>
-      </c>
-      <c r="D36" s="184"/>
-      <c r="E36" s="184"/>
-      <c r="F36" s="184"/>
-    </row>
-    <row r="37" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="C32" s="123" t="s">
+        <v>112</v>
+      </c>
+      <c r="D32" s="124"/>
+      <c r="E32" s="124"/>
+      <c r="F32" s="125"/>
+      <c r="G32" s="54" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="41"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="69"/>
+      <c r="D33" s="70"/>
+      <c r="E33" s="70"/>
+      <c r="F33" s="71"/>
+      <c r="G33" s="33"/>
+    </row>
+    <row r="34" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="42"/>
+      <c r="B34" s="43"/>
+      <c r="C34" s="178"/>
+      <c r="D34" s="178"/>
+      <c r="E34" s="178"/>
+      <c r="F34" s="178"/>
+      <c r="G34" s="44"/>
+    </row>
+    <row r="35" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A35" s="63"/>
+      <c r="B35" s="61" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="186" t="s">
+        <v>95</v>
+      </c>
+      <c r="D35" s="187"/>
+      <c r="E35" s="187"/>
+      <c r="F35" s="188"/>
+      <c r="G35" s="62" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="59" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36" s="60"/>
+      <c r="C36" s="185" t="s">
+        <v>94</v>
+      </c>
+      <c r="D36" s="185"/>
+      <c r="E36" s="185"/>
+      <c r="F36" s="185"/>
+      <c r="G36" s="2"/>
+    </row>
+    <row r="37" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A37" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
-    </row>
-    <row r="38" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
+      <c r="G37" s="2"/>
+    </row>
+    <row r="38" spans="1:7" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A38" s="2" t="s">
         <v>14</v>
       </c>
@@ -3370,21 +3775,10 @@
       </c>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="C25:F25"/>
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="C20:F20"/>
     <mergeCell ref="C8:F8"/>
@@ -3401,6 +3795,18 @@
     <mergeCell ref="C26:F26"/>
     <mergeCell ref="C27:F27"/>
     <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C32:F32"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5">

</xml_diff>